<commit_message>
update with radiometric uncertainty repo
</commit_message>
<xml_diff>
--- a/SAR/Mercedes/TP5 mecanismos/results.xlsx
+++ b/SAR/Mercedes/TP5 mecanismos/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,20 +456,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>laguna</t>
+          <t>laguna2</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-18.64462089538574</v>
+        <v>-18.20027160644531</v>
       </c>
       <c r="D2" t="n">
-        <v>-23.37528038024902</v>
+        <v>-22.99054908752441</v>
       </c>
       <c r="E2" t="n">
-        <v>-19.45305824279785</v>
+        <v>-18.93698883056641</v>
       </c>
       <c r="F2" t="n">
-        <v>-17.71951866149902</v>
+        <v>-17.57296180725098</v>
       </c>
     </row>
     <row r="3">
@@ -480,20 +480,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>juncal</t>
+          <t>laguna1</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-5.607793807983398</v>
+        <v>-18.87930488586426</v>
       </c>
       <c r="D3" t="n">
-        <v>-8.140951156616211</v>
+        <v>-24.00530624389648</v>
       </c>
       <c r="E3" t="n">
-        <v>-8.629714965820312</v>
+        <v>-19.83075904846191</v>
       </c>
       <c r="F3" t="n">
-        <v>-4.35255765914917</v>
+        <v>-18.04147338867188</v>
       </c>
     </row>
     <row r="4">
@@ -504,20 +504,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ciudad</t>
+          <t>juncal2</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-2.529046058654785</v>
+        <v>-4.496796607971191</v>
       </c>
       <c r="D4" t="n">
-        <v>-3.007768630981445</v>
+        <v>-9.363312721252441</v>
       </c>
       <c r="E4" t="n">
-        <v>-3.900567293167114</v>
+        <v>-5.620543956756592</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2945488691329956</v>
+        <v>-3.586736679077148</v>
       </c>
     </row>
     <row r="5">
@@ -528,20 +528,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bosque</t>
+          <t>juncal1</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-6.699508666992188</v>
+        <v>-7.387124061584473</v>
       </c>
       <c r="D5" t="n">
-        <v>-9.593179702758789</v>
+        <v>-8.307149887084961</v>
       </c>
       <c r="E5" t="n">
-        <v>-8.126934051513672</v>
+        <v>-10.67955017089844</v>
       </c>
       <c r="F5" t="n">
-        <v>-5.150150775909424</v>
+        <v>-5.034629821777344</v>
       </c>
     </row>
     <row r="6">
@@ -552,20 +552,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pastizal</t>
+          <t>ciudad2</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-8.368853569030762</v>
+        <v>-3.132599353790283</v>
       </c>
       <c r="D6" t="n">
-        <v>-13.23326683044434</v>
+        <v>-6.273908138275146</v>
       </c>
       <c r="E6" t="n">
-        <v>-9.377289772033691</v>
+        <v>-4.145248413085938</v>
       </c>
       <c r="F6" t="n">
-        <v>-7.495739459991455</v>
+        <v>-1.787373423576355</v>
       </c>
     </row>
     <row r="7">
@@ -576,20 +576,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pajonal</t>
+          <t>ciudad1</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-8.090002059936523</v>
+        <v>1.000223398208618</v>
       </c>
       <c r="D7" t="n">
-        <v>-11.30326747894287</v>
+        <v>-2.134681224822998</v>
       </c>
       <c r="E7" t="n">
-        <v>-11.72356986999512</v>
+        <v>-0.3676701188087463</v>
       </c>
       <c r="F7" t="n">
-        <v>-7.225945472717285</v>
+        <v>2.193089008331299</v>
       </c>
     </row>
     <row r="8">
@@ -600,356 +600,1196 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pradera</t>
+          <t>bosque2</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-10.26866722106934</v>
+        <v>-7.966724395751953</v>
       </c>
       <c r="D8" t="n">
-        <v>-13.27789306640625</v>
+        <v>-12.02756690979004</v>
       </c>
       <c r="E8" t="n">
-        <v>-11.51257705688477</v>
+        <v>-8.991159439086914</v>
       </c>
       <c r="F8" t="n">
-        <v>-8.897704124450684</v>
+        <v>-6.924130439758301</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2008-05</t>
+          <t>2007-03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>laguna</t>
+          <t>bosque1</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-18.3535041809082</v>
+        <v>-5.179946899414062</v>
       </c>
       <c r="D9" t="n">
-        <v>-8.865262031555176</v>
+        <v>-10.03821754455566</v>
       </c>
       <c r="E9" t="n">
-        <v>-19.52737045288086</v>
+        <v>-6.119009017944336</v>
       </c>
       <c r="F9" t="n">
-        <v>-6.478883743286133</v>
+        <v>-4.309710502624512</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2008-05</t>
+          <t>2007-03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>juncal</t>
+          <t>pastizal2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-13.46590137481689</v>
+        <v>-7.56800651550293</v>
       </c>
       <c r="D10" t="n">
-        <v>-13.53573226928711</v>
+        <v>-12.74804210662842</v>
       </c>
       <c r="E10" t="n">
-        <v>-14.56920146942139</v>
+        <v>-8.604469299316406</v>
       </c>
       <c r="F10" t="n">
-        <v>-11.55817413330078</v>
+        <v>-6.830926895141602</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2008-05</t>
+          <t>2007-03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ciudad</t>
+          <t>pastizal1</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-2.815749883651733</v>
+        <v>-8.753137588500977</v>
       </c>
       <c r="D11" t="n">
-        <v>-3.801458835601807</v>
+        <v>-14.71619129180908</v>
       </c>
       <c r="E11" t="n">
-        <v>-3.963114976882935</v>
+        <v>-9.648994445800781</v>
       </c>
       <c r="F11" t="n">
-        <v>-1.119440197944641</v>
+        <v>-8.073807716369629</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2008-05</t>
+          <t>2007-03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bosque</t>
+          <t>pajonal2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-9.523708343505859</v>
+        <v>-15.55998706817627</v>
       </c>
       <c r="D12" t="n">
-        <v>-14.96492862701416</v>
+        <v>-15.35856246948242</v>
       </c>
       <c r="E12" t="n">
-        <v>-10.34043884277344</v>
+        <v>-17.10578727722168</v>
       </c>
       <c r="F12" t="n">
-        <v>-8.629903793334961</v>
+        <v>-13.22656631469727</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2008-05</t>
+          <t>2007-03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>pastizal</t>
+          <t>pajonal1</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-12.37244129180908</v>
+        <v>-7.596557140350342</v>
       </c>
       <c r="D13" t="n">
-        <v>-16.3298454284668</v>
+        <v>-13.53971576690674</v>
       </c>
       <c r="E13" t="n">
-        <v>-13.33396053314209</v>
+        <v>-8.277396202087402</v>
       </c>
       <c r="F13" t="n">
-        <v>-11.02200126647949</v>
+        <v>-6.89926815032959</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2008-05</t>
+          <t>2007-03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>pajonal</t>
+          <t>pradera2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-9.281747817993164</v>
+        <v>-10.10407638549805</v>
       </c>
       <c r="D14" t="n">
-        <v>-13.28637981414795</v>
+        <v>-13.30384159088135</v>
       </c>
       <c r="E14" t="n">
-        <v>-10.63850784301758</v>
+        <v>-11.34348011016846</v>
       </c>
       <c r="F14" t="n">
-        <v>-8.250704765319824</v>
+        <v>-8.769017219543457</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2008-05</t>
+          <t>2007-03</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>pradera</t>
+          <t>pradera1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-10.69509696960449</v>
+        <v>-10.49315452575684</v>
       </c>
       <c r="D15" t="n">
-        <v>-14.79231929779053</v>
+        <v>-13.29974746704102</v>
       </c>
       <c r="E15" t="n">
-        <v>-11.72370052337646</v>
+        <v>-11.81579113006592</v>
       </c>
       <c r="F15" t="n">
-        <v>-9.567185401916504</v>
+        <v>-9.101332664489746</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2005-09</t>
+          <t>2008-05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>laguna</t>
+          <t>laguna2</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-22.07948684692383</v>
+        <v>-6.085638523101807</v>
       </c>
       <c r="D16" t="n">
-        <v>-25.60756492614746</v>
+        <v>-11.24680328369141</v>
       </c>
       <c r="E16" t="n">
-        <v>-23.02231025695801</v>
+        <v>-6.756853103637695</v>
       </c>
       <c r="F16" t="n">
-        <v>-20.44241714477539</v>
+        <v>-5.090959072113037</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2005-09</t>
+          <t>2008-05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>juncal</t>
+          <t>laguna1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-2.826524019241333</v>
+        <v>-19.25679397583008</v>
       </c>
       <c r="D17" t="n">
-        <v>-7.612154483795166</v>
+        <v>-25.81026077270508</v>
       </c>
       <c r="E17" t="n">
-        <v>-3.87132740020752</v>
+        <v>-19.98477172851562</v>
       </c>
       <c r="F17" t="n">
-        <v>-2.026532173156738</v>
+        <v>-18.65017700195312</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2005-09</t>
+          <t>2008-05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ciudad</t>
+          <t>juncal2</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-3.496307134628296</v>
+        <v>-10.36447143554688</v>
       </c>
       <c r="D18" t="n">
-        <v>-5.374110221862793</v>
+        <v>-12.9271297454834</v>
       </c>
       <c r="E18" t="n">
-        <v>-4.606334686279297</v>
+        <v>-13.32758140563965</v>
       </c>
       <c r="F18" t="n">
-        <v>-1.969815373420715</v>
+        <v>-8.848360061645508</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2005-09</t>
+          <t>2008-05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>bosque</t>
+          <t>juncal1</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-9.238754272460938</v>
+        <v>-14.24045562744141</v>
       </c>
       <c r="D19" t="n">
-        <v>-11.29096508026123</v>
+        <v>-19.21672248840332</v>
       </c>
       <c r="E19" t="n">
-        <v>-10.28603649139404</v>
+        <v>-15.42533874511719</v>
       </c>
       <c r="F19" t="n">
-        <v>-8.018179893493652</v>
+        <v>-13.29689598083496</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2005-09</t>
+          <t>2008-05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>pastizal</t>
+          <t>ciudad2</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>-9.332324981689453</v>
+        <v>-3.288486003875732</v>
       </c>
       <c r="D20" t="n">
-        <v>-12.3592414855957</v>
+        <v>-6.117382049560547</v>
       </c>
       <c r="E20" t="n">
-        <v>-10.67838096618652</v>
+        <v>-4.163394927978516</v>
       </c>
       <c r="F20" t="n">
-        <v>-7.859105587005615</v>
+        <v>-1.976343154907227</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2005-09</t>
+          <t>2008-05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>pajonal</t>
+          <t>ciudad1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>-8.425740242004395</v>
+        <v>0.006593325641006231</v>
       </c>
       <c r="D21" t="n">
-        <v>-12.57552719116211</v>
+        <v>-2.627482414245605</v>
       </c>
       <c r="E21" t="n">
-        <v>-9.246458053588867</v>
+        <v>-2.185041666030884</v>
       </c>
       <c r="F21" t="n">
-        <v>-7.432695388793945</v>
+        <v>1.504326462745667</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>2008-05</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>bosque2</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>-9.116313934326172</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-15.07862281799316</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-9.850048065185547</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-8.394692420959473</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2008-05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>bosque1</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>-9.893766403198242</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-15.15861415863037</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-10.62870788574219</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-9.143157005310059</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2008-05</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>pastizal2</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>-13.11543369293213</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-17.26565933227539</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-13.88240432739258</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-12.40037727355957</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2008-05</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>pastizal1</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>-11.47298908233643</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-16.47182464599609</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-12.73469829559326</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-10.61807823181152</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2008-05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pajonal2</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>-11.78947067260742</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-15.14098930358887</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-13.15127468109131</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-10.67467784881592</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2008-05</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>pajonal1</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>-8.712448120117188</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-14.20358657836914</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-9.568645477294922</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-7.891593933105469</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2008-05</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>pradera2</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>-10.83851337432861</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-14.6130542755127</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-11.72629451751709</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-9.514616966247559</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2008-05</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>pradera1</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>-10.41476154327393</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-15.17602920532227</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-11.711181640625</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-9.619985580444336</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>2005-09</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>pradera</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>-9.682312965393066</v>
-      </c>
-      <c r="D22" t="n">
-        <v>-13.78495979309082</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-10.65299415588379</v>
-      </c>
-      <c r="F22" t="n">
-        <v>-8.486473083496094</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>laguna2</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>-20.18142318725586</v>
+      </c>
+      <c r="D30" t="n">
+        <v>-26.90413665771484</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-20.67390823364258</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-19.37871360778809</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>laguna1</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>-22.76121139526367</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-29.65431213378906</v>
+      </c>
+      <c r="E31" t="n">
+        <v>-23.42985343933105</v>
+      </c>
+      <c r="F31" t="n">
+        <v>-22.19841766357422</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>juncal2</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>-3.314886093139648</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-7.9775071144104</v>
+      </c>
+      <c r="E32" t="n">
+        <v>-4.463032722473145</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-2.352165222167969</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>juncal1</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>-2.528265953063965</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-7.688146114349365</v>
+      </c>
+      <c r="E33" t="n">
+        <v>-3.364145278930664</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-1.808178663253784</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ciudad2</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>-3.906062602996826</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-6.196710586547852</v>
+      </c>
+      <c r="E34" t="n">
+        <v>-4.847587108612061</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-2.883235454559326</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ciudad1</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>-1.488417267799377</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-4.959847450256348</v>
+      </c>
+      <c r="E35" t="n">
+        <v>-2.699109554290771</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-0.5722344517707825</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>bosque2</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>-8.103504180908203</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-10.63125419616699</v>
+      </c>
+      <c r="E36" t="n">
+        <v>-9.224356651306152</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-6.352993011474609</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>bosque1</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>-9.904767036437988</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-15.94638919830322</v>
+      </c>
+      <c r="E37" t="n">
+        <v>-10.87000942230225</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-9.246724128723145</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>pastizal2</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>-7.611145496368408</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-12.23497200012207</v>
+      </c>
+      <c r="E38" t="n">
+        <v>-8.752192497253418</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-6.649360179901123</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>pastizal1</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>-10.23703002929688</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-15.47768020629883</v>
+      </c>
+      <c r="E39" t="n">
+        <v>-11.06675338745117</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-9.317633628845215</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>pajonal2</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>-7.543488025665283</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-11.59168434143066</v>
+      </c>
+      <c r="E40" t="n">
+        <v>-8.399115562438965</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-6.193635940551758</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>pajonal1</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>-8.649397850036621</v>
+      </c>
+      <c r="D41" t="n">
+        <v>-14.0401439666748</v>
+      </c>
+      <c r="E41" t="n">
+        <v>-9.582934379577637</v>
+      </c>
+      <c r="F41" t="n">
+        <v>-7.801270008087158</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>pradera2</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>-9.21690559387207</v>
+      </c>
+      <c r="D42" t="n">
+        <v>-13.82613182067871</v>
+      </c>
+      <c r="E42" t="n">
+        <v>-10.05254554748535</v>
+      </c>
+      <c r="F42" t="n">
+        <v>-8.187446594238281</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2005-09</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>pradera1</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>-10.52472114562988</v>
+      </c>
+      <c r="D43" t="n">
+        <v>-15.31142044067383</v>
+      </c>
+      <c r="E43" t="n">
+        <v>-11.58476257324219</v>
+      </c>
+      <c r="F43" t="n">
+        <v>-9.774333953857422</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>laguna2</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>-7.974919319152832</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-13.25228881835938</v>
+      </c>
+      <c r="E44" t="n">
+        <v>-8.990005493164062</v>
+      </c>
+      <c r="F44" t="n">
+        <v>-7.315741539001465</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>laguna1</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>-17.9128246307373</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-23.81568145751953</v>
+      </c>
+      <c r="E45" t="n">
+        <v>-18.64717674255371</v>
+      </c>
+      <c r="F45" t="n">
+        <v>-17.11466026306152</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>juncal2</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>-7.97822380065918</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-12.59041881561279</v>
+      </c>
+      <c r="E46" t="n">
+        <v>-9.109485626220703</v>
+      </c>
+      <c r="F46" t="n">
+        <v>-7.189682006835938</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>juncal1</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>-9.391834259033203</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-14.91885662078857</v>
+      </c>
+      <c r="E47" t="n">
+        <v>-10.16274356842041</v>
+      </c>
+      <c r="F47" t="n">
+        <v>-8.758623123168945</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ciudad2</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>-3.256146907806396</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-6.226149559020996</v>
+      </c>
+      <c r="E48" t="n">
+        <v>-4.359598636627197</v>
+      </c>
+      <c r="F48" t="n">
+        <v>-2.156034469604492</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ciudad1</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>0.2126081585884094</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-1.886275410652161</v>
+      </c>
+      <c r="E49" t="n">
+        <v>-2.10103964805603</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1.345380663871765</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>bosque2</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>-7.165221214294434</v>
+      </c>
+      <c r="D50" t="n">
+        <v>-11.46867656707764</v>
+      </c>
+      <c r="E50" t="n">
+        <v>-8.534580230712891</v>
+      </c>
+      <c r="F50" t="n">
+        <v>-6.042494773864746</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>bosque1</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>-8.256912231445312</v>
+      </c>
+      <c r="D51" t="n">
+        <v>-14.26501178741455</v>
+      </c>
+      <c r="E51" t="n">
+        <v>-8.948013305664062</v>
+      </c>
+      <c r="F51" t="n">
+        <v>-7.564717292785645</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>pastizal2</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>-8.035396575927734</v>
+      </c>
+      <c r="D52" t="n">
+        <v>-13.17895889282227</v>
+      </c>
+      <c r="E52" t="n">
+        <v>-9.150508880615234</v>
+      </c>
+      <c r="F52" t="n">
+        <v>-7.130620002746582</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>pastizal1</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>-11.10786819458008</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-16.78155136108398</v>
+      </c>
+      <c r="E53" t="n">
+        <v>-11.94093894958496</v>
+      </c>
+      <c r="F53" t="n">
+        <v>-10.30178070068359</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>pajonal2</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>-9.426488876342773</v>
+      </c>
+      <c r="D54" t="n">
+        <v>-14.86589241027832</v>
+      </c>
+      <c r="E54" t="n">
+        <v>-10.14615249633789</v>
+      </c>
+      <c r="F54" t="n">
+        <v>-8.789090156555176</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>pajonal1</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>-7.896602630615234</v>
+      </c>
+      <c r="D55" t="n">
+        <v>-12.99306297302246</v>
+      </c>
+      <c r="E55" t="n">
+        <v>-8.800676345825195</v>
+      </c>
+      <c r="F55" t="n">
+        <v>-7.031599998474121</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>pradera2</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>-8.969446182250977</v>
+      </c>
+      <c r="D56" t="n">
+        <v>-14.11079978942871</v>
+      </c>
+      <c r="E56" t="n">
+        <v>-10.10315704345703</v>
+      </c>
+      <c r="F56" t="n">
+        <v>-8.101731300354004</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2008-03</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>pradera1</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>-9.756026268005371</v>
+      </c>
+      <c r="D57" t="n">
+        <v>-13.21043014526367</v>
+      </c>
+      <c r="E57" t="n">
+        <v>-10.75146484375</v>
+      </c>
+      <c r="F57" t="n">
+        <v>-8.021699905395508</v>
       </c>
     </row>
   </sheetData>

</xml_diff>